<commit_message>
feat: Update FinancialReportsPage to support Excel export with template integration
</commit_message>
<xml_diff>
--- a/client/public/templates/Audited Accounts 2425.xlsx
+++ b/client/public/templates/Audited Accounts 2425.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20361"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\E Drive\University Project\L3S1\LankaCapital_ERP_Web\client\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94E53E6F-A3EA-4D12-AFA5-D324F08EB400}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{193420E6-1C9F-4B43-AF6D-66B78887498E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="12072" windowHeight="4512" tabRatio="705" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1957,6 +1957,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:I8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2002,9 +2003,8 @@
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="144" t="str">
-        <f>+Working!A20</f>
-        <v>Furniture &amp; Fittings</v>
+      <c r="A4" t="s">
+        <v>116</v>
       </c>
       <c r="B4" s="145">
         <v>45385</v>
@@ -2013,7 +2013,6 @@
         <v>5</v>
       </c>
       <c r="D4" s="146">
-        <f>+Working!B20</f>
         <v>153700</v>
       </c>
       <c r="E4" s="145">
@@ -2030,9 +2029,8 @@
       <c r="I4" s="176"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="144" t="str">
-        <f>+Working!A21</f>
-        <v>Office Equipment</v>
+      <c r="A5" t="s">
+        <v>170</v>
       </c>
       <c r="B5" s="145">
         <v>45388</v>
@@ -2041,7 +2039,6 @@
         <v>5</v>
       </c>
       <c r="D5" s="146">
-        <f>+Working!B21</f>
         <v>4600</v>
       </c>
       <c r="E5" s="145">
@@ -2081,6 +2078,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:AMD67"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2546,6 +2544,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <sheetPr codeName="Sheet11"/>
   <dimension ref="A1:K54"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
@@ -3161,6 +3160,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2A291A8-AC8E-4BB6-A21B-06A29BC55837}">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A2:D34"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3294,10 +3294,12 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
-        <v>116</v>
+      <c r="A20" t="str">
+        <f>+PPE!A4</f>
+        <v>Furniture &amp; Fittings</v>
       </c>
       <c r="B20" s="175">
+        <f>+PPE!D4</f>
         <v>153700</v>
       </c>
       <c r="C20">
@@ -3305,10 +3307,12 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>170</v>
+      <c r="A21" t="str">
+        <f>+PPE!A5</f>
+        <v>Office Equipment</v>
       </c>
       <c r="B21" s="175">
+        <f>+PPE!D5</f>
         <v>4600</v>
       </c>
       <c r="C21">
@@ -3486,6 +3490,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:J51"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3956,6 +3961,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:G24"/>
   <sheetFormatPr defaultColWidth="8.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
@@ -4130,6 +4136,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:ALX51"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
@@ -43538,6 +43545,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:J23"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
@@ -43782,6 +43790,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:I43"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
@@ -44133,6 +44142,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <sheetPr codeName="Sheet8"/>
   <dimension ref="A1:I35"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>
@@ -44553,6 +44563,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <sheetPr codeName="Sheet9"/>
   <dimension ref="A1:AMD52"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>